<commit_message>
rerun annotation data scripts
</commit_message>
<xml_diff>
--- a/annotation/Species_list_vs_CATAMI_2023_07.xlsx
+++ b/annotation/Species_list_vs_CATAMI_2023_07.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26626"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjansen\Desktop\science\SouthernOceanBiodiversityMapping\ARC_Data\annotation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037E662F-FA1F-4BF6-8ADD-3DA130A8C9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5020AF6-DE26-418B-8A98-F2B7D84C532D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15030" yWindow="-18120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15060" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER_naming" sheetId="1" r:id="rId1"/>
@@ -1885,7 +1885,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1905,9 +1905,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1915,9 +1912,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2320,7 +2314,7 @@
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.109375" customWidth="1"/>
-    <col min="5" max="5" width="68.44140625" style="16" customWidth="1"/>
+    <col min="5" max="5" width="68.44140625" style="14" customWidth="1"/>
     <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.109375" style="2" customWidth="1"/>
@@ -2354,7 +2348,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>498</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -2425,7 +2419,7 @@
       <c r="D2" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="14" t="s">
         <v>570</v>
       </c>
       <c r="F2" s="2">
@@ -2466,7 +2460,7 @@
       <c r="D3" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="14" t="s">
         <v>571</v>
       </c>
       <c r="F3" s="2">
@@ -2510,7 +2504,7 @@
       <c r="D4" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="14" t="s">
         <v>572</v>
       </c>
       <c r="F4" s="2">
@@ -2551,7 +2545,7 @@
       <c r="D5" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="14" t="s">
         <v>573</v>
       </c>
       <c r="F5" s="2">
@@ -2588,7 +2582,7 @@
       <c r="D6" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="14" t="s">
         <v>574</v>
       </c>
       <c r="F6" s="2">
@@ -2641,7 +2635,7 @@
       <c r="D7" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="14" t="s">
         <v>575</v>
       </c>
       <c r="F7" s="2">
@@ -2685,10 +2679,10 @@
       <c r="D8" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="13" t="s">
         <v>575</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="9">
         <v>372</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -2735,10 +2729,10 @@
       <c r="D9" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="13" t="s">
         <v>575</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="9">
         <v>372</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -2779,7 +2773,7 @@
       <c r="D10" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="14" t="s">
         <v>576</v>
       </c>
       <c r="F10" s="2">
@@ -2823,7 +2817,7 @@
       <c r="D11" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="14" t="s">
         <v>577</v>
       </c>
       <c r="F11" s="2">
@@ -2867,7 +2861,7 @@
       <c r="D12" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="14" t="s">
         <v>578</v>
       </c>
       <c r="F12" s="2">
@@ -2911,7 +2905,7 @@
       <c r="D13" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="11" t="s">
         <v>506</v>
       </c>
       <c r="F13" s="2">
@@ -2961,10 +2955,10 @@
       <c r="D14" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="13" t="s">
         <v>579</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="9">
         <v>447</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -3005,10 +2999,10 @@
       <c r="D15" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="13" t="s">
         <v>579</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="9">
         <v>447</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -3049,10 +3043,10 @@
       <c r="D16" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="13" t="s">
         <v>579</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="9">
         <v>447</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -3093,10 +3087,10 @@
       <c r="D17" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="13" t="s">
         <v>579</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="9">
         <v>447</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -3146,7 +3140,7 @@
       <c r="D18" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="14" t="s">
         <v>580</v>
       </c>
       <c r="F18" s="2">
@@ -3190,7 +3184,7 @@
       <c r="D19" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="14" t="s">
         <v>581</v>
       </c>
       <c r="F19" s="2">
@@ -3234,7 +3228,7 @@
       <c r="D20" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="14" t="s">
         <v>582</v>
       </c>
       <c r="F20" s="2">
@@ -3278,10 +3272,10 @@
       <c r="D21" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="13" t="s">
         <v>583</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="9">
         <v>446</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -3322,10 +3316,10 @@
       <c r="D22" s="2" t="s">
         <v>485</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="13" t="s">
         <v>583</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="9">
         <v>446</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -3366,7 +3360,7 @@
       <c r="D23" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="E23" s="16" t="s">
+      <c r="E23" s="14" t="s">
         <v>584</v>
       </c>
       <c r="F23" s="2">
@@ -3410,10 +3404,10 @@
       <c r="D24" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="13" t="s">
         <v>585</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="9">
         <v>451</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -3454,7 +3448,7 @@
       <c r="D25" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="14" t="s">
         <v>586</v>
       </c>
       <c r="F25" s="2">
@@ -3498,7 +3492,7 @@
       <c r="D26" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E26" s="16" t="s">
+      <c r="E26" s="14" t="s">
         <v>587</v>
       </c>
       <c r="F26" s="2">
@@ -3539,10 +3533,10 @@
       <c r="D27" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="11" t="s">
         <v>502</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="2">
         <v>14969</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -3589,7 +3583,7 @@
       <c r="D28" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="11" t="s">
         <v>503</v>
       </c>
       <c r="F28" s="2">
@@ -3642,10 +3636,10 @@
       <c r="D29" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="11" t="s">
         <v>500</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="2">
         <v>14968</v>
       </c>
       <c r="G29" s="3" t="s">
@@ -3692,10 +3686,10 @@
       <c r="D30" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="F30" s="10">
+      <c r="F30" s="9">
         <v>14968</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -3742,7 +3736,7 @@
       <c r="D31" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="11" t="s">
         <v>501</v>
       </c>
       <c r="F31" s="2">
@@ -3795,10 +3789,10 @@
       <c r="D32" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="11" t="s">
         <v>511</v>
       </c>
-      <c r="F32" s="9">
+      <c r="F32" s="2">
         <v>533</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -3848,10 +3842,10 @@
       <c r="D33" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="E33" s="12" t="s">
         <v>511</v>
       </c>
-      <c r="F33" s="10">
+      <c r="F33" s="9">
         <v>533</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -3910,10 +3904,10 @@
       <c r="D34" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="12" t="s">
         <v>511</v>
       </c>
-      <c r="F34" s="10">
+      <c r="F34" s="9">
         <v>533</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -3963,10 +3957,10 @@
       <c r="D35" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="F35" s="10">
+      <c r="F35" s="9">
         <v>524</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -4015,10 +4009,10 @@
       <c r="D36" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="E36" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="F36" s="10">
+      <c r="F36" s="9">
         <v>524</v>
       </c>
       <c r="G36" s="3" t="s">
@@ -4068,7 +4062,7 @@
       <c r="D37" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="11" t="s">
         <v>512</v>
       </c>
       <c r="F37" s="2">
@@ -4121,10 +4115,10 @@
       <c r="D38" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="E38" s="14" t="s">
+      <c r="E38" s="12" t="s">
         <v>513</v>
       </c>
-      <c r="F38" s="10">
+      <c r="F38" s="9">
         <v>536</v>
       </c>
       <c r="G38" s="3" t="s">
@@ -4174,10 +4168,10 @@
       <c r="D39" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E39" s="12" t="s">
         <v>513</v>
       </c>
-      <c r="F39" s="10">
+      <c r="F39" s="9">
         <v>536</v>
       </c>
       <c r="G39" s="3" t="s">
@@ -4227,10 +4221,10 @@
       <c r="D40" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="E40" s="14" t="s">
+      <c r="E40" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="F40" s="10">
+      <c r="F40" s="9">
         <v>531</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -4289,10 +4283,10 @@
       <c r="D41" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="11" t="s">
         <v>510</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="2">
         <v>531</v>
       </c>
       <c r="G41" s="3" t="s">
@@ -4342,10 +4336,10 @@
       <c r="D42" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="E42" s="14" t="s">
+      <c r="E42" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="F42" s="10">
+      <c r="F42" s="9">
         <v>531</v>
       </c>
       <c r="G42" s="3" t="s">
@@ -4395,10 +4389,10 @@
       <c r="D43" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="E43" s="14" t="s">
+      <c r="E43" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="F43" s="10">
+      <c r="F43" s="9">
         <v>531</v>
       </c>
       <c r="G43" s="3" t="s">
@@ -4448,10 +4442,10 @@
       <c r="D44" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="E44" s="14" t="s">
+      <c r="E44" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="F44" s="10">
+      <c r="F44" s="9">
         <v>531</v>
       </c>
       <c r="G44" s="3" t="s">
@@ -4510,10 +4504,10 @@
       <c r="D45" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="E45" s="14" t="s">
+      <c r="E45" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="F45" s="10">
+      <c r="F45" s="9">
         <v>15005</v>
       </c>
       <c r="G45" s="3" t="s">
@@ -4563,7 +4557,7 @@
       <c r="D46" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="E46" s="12" t="s">
+      <c r="E46" s="11" t="s">
         <v>509</v>
       </c>
       <c r="F46" s="2">
@@ -4615,10 +4609,10 @@
       <c r="D47" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="E47" s="11" t="s">
         <v>508</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="2">
         <v>15005</v>
       </c>
       <c r="G47" s="3" t="s">
@@ -4668,10 +4662,10 @@
       <c r="D48" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="E48" s="14" t="s">
+      <c r="E48" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="F48" s="10">
+      <c r="F48" s="9">
         <v>15005</v>
       </c>
       <c r="G48" s="3" t="s">
@@ -4721,10 +4715,10 @@
       <c r="D49" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="E49" s="14" t="s">
+      <c r="E49" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="F49" s="10">
+      <c r="F49" s="9">
         <v>15005</v>
       </c>
       <c r="G49" s="3" t="s">
@@ -4774,7 +4768,7 @@
       <c r="D50" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="E50" s="11" t="s">
         <v>514</v>
       </c>
       <c r="F50" s="2">
@@ -4827,8 +4821,8 @@
       <c r="D51" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="E51" s="19"/>
-      <c r="F51" s="20"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="18"/>
       <c r="J51">
         <v>5</v>
       </c>
@@ -4858,7 +4852,7 @@
       <c r="D52" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="11" t="s">
         <v>515</v>
       </c>
       <c r="F52" s="2">
@@ -4911,10 +4905,10 @@
       <c r="D53" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E53" s="14" t="s">
+      <c r="E53" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="F53" s="10">
+      <c r="F53" s="9">
         <v>500</v>
       </c>
       <c r="G53" s="3" t="s">
@@ -4952,10 +4946,10 @@
       <c r="D54" t="s">
         <v>249</v>
       </c>
-      <c r="E54" s="14" t="s">
+      <c r="E54" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="F54" s="10">
+      <c r="F54" s="9">
         <v>500</v>
       </c>
       <c r="G54" s="3"/>
@@ -4997,7 +4991,7 @@
       <c r="D55" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E55" s="16" t="s">
+      <c r="E55" s="14" t="s">
         <v>560</v>
       </c>
       <c r="F55" s="2">
@@ -5041,10 +5035,10 @@
       <c r="D56" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="E56" s="14" t="s">
+      <c r="E56" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="F56" s="10">
+      <c r="F56" s="9">
         <v>500</v>
       </c>
       <c r="G56" s="3" t="s">
@@ -5082,10 +5076,10 @@
       <c r="D57" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="E57" s="14" t="s">
+      <c r="E57" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="F57" s="10">
+      <c r="F57" s="9">
         <v>500</v>
       </c>
       <c r="G57" s="3" t="s">
@@ -5132,10 +5126,10 @@
       <c r="D58" t="s">
         <v>252</v>
       </c>
-      <c r="E58" s="14" t="s">
+      <c r="E58" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="F58" s="10">
+      <c r="F58" s="9">
         <v>500</v>
       </c>
       <c r="G58" s="3"/>
@@ -5177,7 +5171,7 @@
       <c r="D59" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="E59" s="12" t="s">
+      <c r="E59" s="11" t="s">
         <v>505</v>
       </c>
       <c r="F59" s="2">
@@ -5236,7 +5230,7 @@
       <c r="D60" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="E60" s="12" t="s">
+      <c r="E60" s="11" t="s">
         <v>519</v>
       </c>
       <c r="F60" s="2">
@@ -5298,7 +5292,7 @@
       <c r="D61" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="E61" s="12" t="s">
+      <c r="E61" s="11" t="s">
         <v>516</v>
       </c>
       <c r="F61" s="2">
@@ -5360,7 +5354,7 @@
       <c r="D62" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="E62" s="12" t="s">
+      <c r="E62" s="11" t="s">
         <v>517</v>
       </c>
       <c r="F62" s="2">
@@ -5419,7 +5413,7 @@
       <c r="D63" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="E63" s="12" t="s">
+      <c r="E63" s="11" t="s">
         <v>522</v>
       </c>
       <c r="F63" s="2">
@@ -5478,7 +5472,7 @@
       <c r="D64" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="E64" s="12" t="s">
+      <c r="E64" s="11" t="s">
         <v>518</v>
       </c>
       <c r="F64" s="2">
@@ -5537,10 +5531,10 @@
       <c r="D65" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="E65" s="14" t="s">
+      <c r="E65" s="12" t="s">
         <v>521</v>
       </c>
-      <c r="F65" s="10">
+      <c r="F65" s="9">
         <v>595</v>
       </c>
       <c r="G65" s="3" t="s">
@@ -5599,10 +5593,10 @@
       <c r="D66" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="E66" s="14" t="s">
+      <c r="E66" s="12" t="s">
         <v>521</v>
       </c>
-      <c r="F66" s="10">
+      <c r="F66" s="9">
         <v>595</v>
       </c>
       <c r="G66" s="3" t="s">
@@ -5661,10 +5655,10 @@
       <c r="D67" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="E67" s="14" t="s">
+      <c r="E67" s="12" t="s">
         <v>521</v>
       </c>
-      <c r="F67" s="10">
+      <c r="F67" s="9">
         <v>595</v>
       </c>
       <c r="G67" s="3" t="s">
@@ -5723,10 +5717,10 @@
       <c r="D68" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E68" s="14" t="s">
+      <c r="E68" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F68" s="10">
+      <c r="F68" s="9">
         <v>7320</v>
       </c>
       <c r="G68" s="3"/>
@@ -5768,10 +5762,10 @@
       <c r="D69" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="E69" s="14" t="s">
+      <c r="E69" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F69" s="10">
+      <c r="F69" s="9">
         <v>7320</v>
       </c>
       <c r="G69" s="3"/>
@@ -5813,10 +5807,10 @@
       <c r="D70" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="E70" s="14" t="s">
+      <c r="E70" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F70" s="10">
+      <c r="F70" s="9">
         <v>7320</v>
       </c>
       <c r="G70" s="3"/>
@@ -5858,10 +5852,10 @@
       <c r="D71" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="E71" s="14" t="s">
+      <c r="E71" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F71" s="10">
+      <c r="F71" s="9">
         <v>7320</v>
       </c>
       <c r="G71" s="3"/>
@@ -5903,10 +5897,10 @@
       <c r="D72" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="E72" s="14" t="s">
+      <c r="E72" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F72" s="10">
+      <c r="F72" s="9">
         <v>7320</v>
       </c>
       <c r="G72" s="3"/>
@@ -5939,10 +5933,10 @@
       <c r="D73" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="E73" s="14" t="s">
+      <c r="E73" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F73" s="10">
+      <c r="F73" s="9">
         <v>7320</v>
       </c>
       <c r="G73" s="3"/>
@@ -5984,10 +5978,10 @@
       <c r="D74" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="E74" s="14" t="s">
+      <c r="E74" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F74" s="10">
+      <c r="F74" s="9">
         <v>7320</v>
       </c>
       <c r="G74" s="3"/>
@@ -6029,10 +6023,10 @@
       <c r="D75" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="E75" s="14" t="s">
+      <c r="E75" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F75" s="10">
+      <c r="F75" s="9">
         <v>7320</v>
       </c>
       <c r="G75" s="3"/>
@@ -6074,7 +6068,7 @@
       <c r="D76" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="E76" s="12" t="s">
+      <c r="E76" s="11" t="s">
         <v>548</v>
       </c>
       <c r="F76" s="2">
@@ -6118,7 +6112,7 @@
       <c r="D77" t="s">
         <v>400</v>
       </c>
-      <c r="E77" s="12" t="s">
+      <c r="E77" s="11" t="s">
         <v>549</v>
       </c>
       <c r="F77" s="2">
@@ -6171,7 +6165,7 @@
       <c r="D78" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="E78" s="12" t="s">
+      <c r="E78" s="11" t="s">
         <v>550</v>
       </c>
       <c r="F78" s="2">
@@ -6221,7 +6215,7 @@
       <c r="D79" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="E79" s="12" t="s">
+      <c r="E79" s="11" t="s">
         <v>551</v>
       </c>
       <c r="F79" s="2">
@@ -6271,10 +6265,10 @@
       <c r="D80" t="s">
         <v>397</v>
       </c>
-      <c r="E80" s="14" t="s">
+      <c r="E80" s="12" t="s">
         <v>557</v>
       </c>
-      <c r="F80" s="10">
+      <c r="F80" s="9">
         <v>459</v>
       </c>
       <c r="G80" s="3" t="s">
@@ -6321,7 +6315,7 @@
       <c r="D81" t="s">
         <v>396</v>
       </c>
-      <c r="E81" s="12" t="s">
+      <c r="E81" s="11" t="s">
         <v>552</v>
       </c>
       <c r="F81" s="2">
@@ -6365,7 +6359,7 @@
       <c r="D82" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="E82" s="12" t="s">
+      <c r="E82" s="11" t="s">
         <v>553</v>
       </c>
       <c r="F82" s="2">
@@ -6409,7 +6403,7 @@
       <c r="D83" t="s">
         <v>393</v>
       </c>
-      <c r="E83" s="12" t="s">
+      <c r="E83" s="11" t="s">
         <v>554</v>
       </c>
       <c r="F83" s="2">
@@ -6462,7 +6456,7 @@
       <c r="D84" t="s">
         <v>394</v>
       </c>
-      <c r="E84" s="12" t="s">
+      <c r="E84" s="11" t="s">
         <v>555</v>
       </c>
       <c r="F84" s="2">
@@ -6515,7 +6509,7 @@
       <c r="D85" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="E85" s="12" t="s">
+      <c r="E85" s="11" t="s">
         <v>556</v>
       </c>
       <c r="F85" s="2">
@@ -6559,10 +6553,10 @@
       <c r="D86" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E86" s="14" t="s">
+      <c r="E86" s="12" t="s">
         <v>557</v>
       </c>
-      <c r="F86" s="10">
+      <c r="F86" s="9">
         <v>459</v>
       </c>
       <c r="G86" s="3" t="s">
@@ -6600,7 +6594,7 @@
       <c r="D87" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="E87" s="12" t="s">
+      <c r="E87" s="11" t="s">
         <v>558</v>
       </c>
       <c r="F87" s="2">
@@ -6644,7 +6638,7 @@
       <c r="D88" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E88" s="12" t="s">
+      <c r="E88" s="11" t="s">
         <v>529</v>
       </c>
       <c r="F88" s="2">
@@ -6694,7 +6688,7 @@
       <c r="D89" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E89" s="12" t="s">
+      <c r="E89" s="11" t="s">
         <v>523</v>
       </c>
       <c r="F89" s="2">
@@ -6747,10 +6741,10 @@
       <c r="D90" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="E90" s="14" t="s">
+      <c r="E90" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F90" s="10">
+      <c r="F90" s="9">
         <v>630</v>
       </c>
       <c r="G90" s="3" t="s">
@@ -6791,10 +6785,10 @@
       <c r="D91" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="E91" s="14" t="s">
+      <c r="E91" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F91" s="10">
+      <c r="F91" s="9">
         <v>630</v>
       </c>
       <c r="G91" s="3" t="s">
@@ -6844,10 +6838,10 @@
       <c r="D92" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="E92" s="14" t="s">
+      <c r="E92" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F92" s="10">
+      <c r="F92" s="9">
         <v>630</v>
       </c>
       <c r="G92" s="3" t="s">
@@ -6888,10 +6882,10 @@
       <c r="D93" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="E93" s="14" t="s">
+      <c r="E93" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F93" s="10">
+      <c r="F93" s="9">
         <v>630</v>
       </c>
       <c r="G93" s="3" t="s">
@@ -6935,10 +6929,10 @@
       <c r="D94" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="E94" s="14" t="s">
+      <c r="E94" s="12" t="s">
         <v>542</v>
       </c>
-      <c r="F94" s="10">
+      <c r="F94" s="9">
         <v>628</v>
       </c>
       <c r="G94" s="3" t="s">
@@ -6979,10 +6973,10 @@
       <c r="D95" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="E95" s="14" t="s">
+      <c r="E95" s="12" t="s">
         <v>542</v>
       </c>
-      <c r="F95" s="10">
+      <c r="F95" s="9">
         <v>628</v>
       </c>
       <c r="G95" s="3" t="s">
@@ -7026,10 +7020,10 @@
       <c r="D96" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="E96" s="14" t="s">
+      <c r="E96" s="12" t="s">
         <v>543</v>
       </c>
-      <c r="F96" s="10">
+      <c r="F96" s="9">
         <v>615</v>
       </c>
       <c r="G96" s="3" t="s">
@@ -7070,10 +7064,10 @@
       <c r="D97" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="E97" s="14" t="s">
+      <c r="E97" s="12" t="s">
         <v>543</v>
       </c>
-      <c r="F97" s="10">
+      <c r="F97" s="9">
         <v>615</v>
       </c>
       <c r="G97" s="3" t="s">
@@ -7114,10 +7108,10 @@
       <c r="D98" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="E98" s="14" t="s">
+      <c r="E98" s="12" t="s">
         <v>544</v>
       </c>
-      <c r="F98" s="10">
+      <c r="F98" s="9">
         <v>609</v>
       </c>
       <c r="G98" s="3" t="s">
@@ -7164,10 +7158,10 @@
       <c r="D99" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="E99" s="14" t="s">
+      <c r="E99" s="12" t="s">
         <v>535</v>
       </c>
-      <c r="F99" s="10">
+      <c r="F99" s="9">
         <v>622</v>
       </c>
       <c r="G99" s="3" t="s">
@@ -7208,7 +7202,7 @@
       <c r="D100" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="E100" s="12" t="s">
+      <c r="E100" s="11" t="s">
         <v>534</v>
       </c>
       <c r="F100" s="2">
@@ -7252,7 +7246,7 @@
       <c r="D101" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="E101" s="12" t="s">
+      <c r="E101" s="11" t="s">
         <v>545</v>
       </c>
       <c r="F101" s="2">
@@ -7305,7 +7299,7 @@
       <c r="D102" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="E102" s="12" t="s">
+      <c r="E102" s="11" t="s">
         <v>546</v>
       </c>
       <c r="F102" s="2">
@@ -7349,7 +7343,7 @@
       <c r="D103" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="E103" s="12" t="s">
+      <c r="E103" s="11" t="s">
         <v>534</v>
       </c>
       <c r="F103" s="2">
@@ -7393,10 +7387,10 @@
       <c r="D104" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="E104" s="14" t="s">
+      <c r="E104" s="12" t="s">
         <v>540</v>
       </c>
-      <c r="F104" s="10">
+      <c r="F104" s="9">
         <v>621</v>
       </c>
       <c r="G104" s="3" t="s">
@@ -7443,7 +7437,7 @@
       <c r="D105" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="E105" s="12" t="s">
+      <c r="E105" s="11" t="s">
         <v>535</v>
       </c>
       <c r="F105" s="2">
@@ -7487,7 +7481,7 @@
       <c r="D106" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="E106" s="12" t="s">
+      <c r="E106" s="11" t="s">
         <v>536</v>
       </c>
       <c r="F106" s="2">
@@ -7531,7 +7525,7 @@
       <c r="D107" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="E107" s="12" t="s">
+      <c r="E107" s="11" t="s">
         <v>537</v>
       </c>
       <c r="F107" s="2">
@@ -7584,7 +7578,7 @@
       <c r="D108" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="E108" s="12" t="s">
+      <c r="E108" s="11" t="s">
         <v>538</v>
       </c>
       <c r="F108" s="2">
@@ -7634,7 +7628,7 @@
       <c r="D109" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="E109" s="12" t="s">
+      <c r="E109" s="11" t="s">
         <v>539</v>
       </c>
       <c r="F109" s="2">
@@ -7684,10 +7678,10 @@
       <c r="D110" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="E110" s="14" t="s">
+      <c r="E110" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F110" s="10">
+      <c r="F110" s="9">
         <v>630</v>
       </c>
       <c r="G110" s="3" t="s">
@@ -7728,10 +7722,10 @@
       <c r="D111" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="E111" s="14" t="s">
+      <c r="E111" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F111" s="10">
+      <c r="F111" s="9">
         <v>630</v>
       </c>
       <c r="G111" s="3" t="s">
@@ -7772,7 +7766,7 @@
       <c r="D112" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="E112" s="12" t="s">
+      <c r="E112" s="11" t="s">
         <v>547</v>
       </c>
       <c r="F112" s="2">
@@ -7816,8 +7810,8 @@
       <c r="D113" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="E113" s="17"/>
-      <c r="F113" s="18"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="16"/>
       <c r="G113" s="3"/>
       <c r="J113">
         <v>36</v>
@@ -7848,8 +7842,8 @@
       <c r="D114" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="E114" s="17"/>
-      <c r="F114" s="18"/>
+      <c r="E114" s="15"/>
+      <c r="F114" s="16"/>
       <c r="G114" s="3"/>
       <c r="J114">
         <v>49</v>
@@ -7880,7 +7874,7 @@
       <c r="D115" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="E115" s="16" t="s">
+      <c r="E115" s="14" t="s">
         <v>561</v>
       </c>
       <c r="F115" s="2">
@@ -7924,7 +7918,7 @@
       <c r="D116" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="E116" s="16" t="s">
+      <c r="E116" s="14" t="s">
         <v>562</v>
       </c>
       <c r="F116" s="2">
@@ -7968,7 +7962,7 @@
       <c r="D117" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E117" s="16" t="s">
+      <c r="E117" s="14" t="s">
         <v>563</v>
       </c>
       <c r="F117" s="2">
@@ -8018,7 +8012,7 @@
       <c r="D118" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="E118" s="16" t="s">
+      <c r="E118" s="14" t="s">
         <v>564</v>
       </c>
       <c r="F118" s="2">
@@ -8062,10 +8056,10 @@
       <c r="D119" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="E119" s="15" t="s">
+      <c r="E119" s="13" t="s">
         <v>562</v>
       </c>
-      <c r="F119" s="10">
+      <c r="F119" s="9">
         <v>638</v>
       </c>
       <c r="G119" s="3" t="s">
@@ -8106,7 +8100,7 @@
       <c r="D120" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="E120" s="16" t="s">
+      <c r="E120" s="14" t="s">
         <v>565</v>
       </c>
       <c r="F120" s="2">
@@ -8150,7 +8144,7 @@
       <c r="D121" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="E121" s="16" t="s">
+      <c r="E121" s="14" t="s">
         <v>566</v>
       </c>
       <c r="F121" s="2">
@@ -8194,7 +8188,7 @@
       <c r="D122" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="E122" s="16" t="s">
+      <c r="E122" s="14" t="s">
         <v>567</v>
       </c>
       <c r="F122" s="2">
@@ -8238,7 +8232,7 @@
       <c r="D123" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="E123" s="16" t="s">
+      <c r="E123" s="14" t="s">
         <v>568</v>
       </c>
       <c r="F123" s="2">
@@ -8282,10 +8276,10 @@
       <c r="D124" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E124" s="15" t="s">
+      <c r="E124" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="F124" s="10">
+      <c r="F124" s="9">
         <v>12825</v>
       </c>
       <c r="G124" s="3"/>
@@ -8318,10 +8312,10 @@
       <c r="D125" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E125" s="15" t="s">
+      <c r="E125" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="F125" s="10">
+      <c r="F125" s="9">
         <v>12825</v>
       </c>
       <c r="G125" s="3"/>
@@ -8354,10 +8348,10 @@
       <c r="D126" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="E126" s="15" t="s">
+      <c r="E126" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="F126" s="10">
+      <c r="F126" s="9">
         <v>12825</v>
       </c>
       <c r="G126" s="3"/>
@@ -8390,10 +8384,10 @@
       <c r="D127" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="E127" s="15" t="s">
+      <c r="E127" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="F127" s="10">
+      <c r="F127" s="9">
         <v>12825</v>
       </c>
       <c r="G127" s="3"/>
@@ -8426,10 +8420,10 @@
       <c r="D128" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E128" s="15" t="s">
+      <c r="E128" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="F128" s="10">
+      <c r="F128" s="9">
         <v>12825</v>
       </c>
       <c r="G128" s="3"/>
@@ -8462,7 +8456,7 @@
       <c r="D129" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E129" s="16" t="s">
+      <c r="E129" s="14" t="s">
         <v>140</v>
       </c>
       <c r="F129" s="2">
@@ -8498,10 +8492,10 @@
       <c r="D130" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E130" s="14" t="s">
+      <c r="E130" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="F130" s="10">
+      <c r="F130" s="9">
         <v>650</v>
       </c>
       <c r="G130" s="3" t="s">
@@ -8557,10 +8551,10 @@
       <c r="D131" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="E131" s="14" t="s">
+      <c r="E131" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="F131" s="10">
+      <c r="F131" s="9">
         <v>650</v>
       </c>
       <c r="G131" s="3" t="s">
@@ -8607,10 +8601,10 @@
       <c r="D132" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="E132" s="14" t="s">
+      <c r="E132" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="F132" s="10">
+      <c r="F132" s="9">
         <v>650</v>
       </c>
       <c r="G132" s="3" t="s">
@@ -8657,7 +8651,7 @@
       <c r="D133" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="E133" s="12" t="s">
+      <c r="E133" s="11" t="s">
         <v>531</v>
       </c>
       <c r="F133" s="2">
@@ -8719,10 +8713,10 @@
       <c r="D134" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="E134" s="14" t="s">
+      <c r="E134" s="12" t="s">
         <v>531</v>
       </c>
-      <c r="F134" s="10">
+      <c r="F134" s="9">
         <v>656</v>
       </c>
       <c r="G134" s="3" t="s">
@@ -8772,7 +8766,7 @@
       <c r="D135" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="E135" s="12" t="s">
+      <c r="E135" s="11" t="s">
         <v>526</v>
       </c>
       <c r="F135" s="2">
@@ -8825,10 +8819,10 @@
       <c r="D136" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="E136" s="14" t="s">
+      <c r="E136" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="F136" s="10">
+      <c r="F136" s="9">
         <v>650</v>
       </c>
       <c r="G136" s="3" t="s">
@@ -8884,10 +8878,10 @@
       <c r="D137" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E137" s="15" t="s">
+      <c r="E137" s="13" t="s">
         <v>562</v>
       </c>
-      <c r="F137" s="10">
+      <c r="F137" s="9">
         <v>638</v>
       </c>
       <c r="G137" s="3" t="s">
@@ -8937,10 +8931,10 @@
       <c r="D138" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="E138" s="14" t="s">
+      <c r="E138" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="F138" s="10">
+      <c r="F138" s="9">
         <v>650</v>
       </c>
       <c r="G138" s="3" t="s">
@@ -9198,10 +9192,10 @@
       <c r="D4" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="2">
         <v>14969</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -9239,10 +9233,10 @@
       <c r="D5" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>14969</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -9324,10 +9318,10 @@
       <c r="D7" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="9">
         <v>14969</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -9365,10 +9359,10 @@
       <c r="D8" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="9">
         <v>14969</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -9447,10 +9441,10 @@
       <c r="D10" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>500</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="9">
         <v>14968</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -9576,10 +9570,10 @@
       <c r="D13" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="9">
         <v>15005</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -9670,10 +9664,10 @@
       <c r="D15" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="9">
         <v>15005</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -9723,10 +9717,10 @@
       <c r="D16" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="2">
         <v>15005</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -9767,10 +9761,10 @@
       <c r="D17" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="9">
         <v>15005</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -9811,10 +9805,10 @@
       <c r="D18" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="9">
         <v>15005</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -9855,10 +9849,10 @@
       <c r="D19" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="9">
         <v>15005</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -9899,10 +9893,10 @@
       <c r="D20" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="9">
         <v>15005</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -9943,10 +9937,10 @@
       <c r="D21" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="9">
         <v>15005</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -9987,10 +9981,10 @@
       <c r="D22" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="9">
         <v>15005</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -10031,10 +10025,10 @@
       <c r="D23" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="9">
         <v>15005</v>
       </c>
       <c r="G23" s="3" t="s">
@@ -10075,10 +10069,10 @@
       <c r="D24" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="9" t="s">
         <v>532</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="9">
         <v>524</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -10119,10 +10113,10 @@
       <c r="D25" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="9" t="s">
         <v>532</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F25" s="9">
         <v>524</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -10163,10 +10157,10 @@
       <c r="D26" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="F26" s="10">
+      <c r="F26" s="9">
         <v>531</v>
       </c>
       <c r="G26" s="3" t="s">
@@ -10207,7 +10201,7 @@
       <c r="D27" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="2" t="s">
         <v>510</v>
       </c>
       <c r="F27" s="2">
@@ -10251,10 +10245,10 @@
       <c r="D28" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="F28" s="10">
+      <c r="F28" s="9">
         <v>531</v>
       </c>
       <c r="G28" s="3" t="s">
@@ -10295,10 +10289,10 @@
       <c r="D29" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="F29" s="10">
+      <c r="F29" s="9">
         <v>531</v>
       </c>
       <c r="G29" s="3" t="s">
@@ -10339,10 +10333,10 @@
       <c r="D30" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="F30" s="10">
+      <c r="F30" s="9">
         <v>531</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -10383,7 +10377,7 @@
       <c r="D31" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="2" t="s">
         <v>511</v>
       </c>
       <c r="F31" s="2">
@@ -10427,10 +10421,10 @@
       <c r="D32" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="F32" s="10">
+      <c r="F32" s="9">
         <v>533</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -10471,10 +10465,10 @@
       <c r="D33" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="F33" s="10">
+      <c r="F33" s="9">
         <v>533</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -10524,10 +10518,10 @@
       <c r="D34" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E34" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="F34" s="10">
+      <c r="F34" s="9">
         <v>533</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -10568,10 +10562,10 @@
       <c r="D35" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="F35" s="10">
+      <c r="F35" s="9">
         <v>533</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -10612,7 +10606,7 @@
       <c r="D36" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="2" t="s">
         <v>512</v>
       </c>
       <c r="F36" s="2">
@@ -10656,10 +10650,10 @@
       <c r="D37" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="9" t="s">
         <v>513</v>
       </c>
-      <c r="F37" s="10">
+      <c r="F37" s="9">
         <v>536</v>
       </c>
       <c r="G37" s="3" t="s">
@@ -10700,10 +10694,10 @@
       <c r="D38" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="9" t="s">
         <v>513</v>
       </c>
-      <c r="F38" s="10">
+      <c r="F38" s="9">
         <v>536</v>
       </c>
       <c r="G38" s="3" t="s">
@@ -10744,7 +10738,7 @@
       <c r="D39" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="2" t="s">
         <v>514</v>
       </c>
       <c r="F39" s="2">
@@ -10788,7 +10782,7 @@
       <c r="D40" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="2" t="s">
         <v>515</v>
       </c>
       <c r="F40" s="2">
@@ -11134,10 +11128,10 @@
       <c r="D48" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="E48" s="10" t="s">
+      <c r="E48" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="F48" s="10">
+      <c r="F48" s="9">
         <v>595</v>
       </c>
       <c r="G48" s="3" t="s">
@@ -11178,10 +11172,10 @@
       <c r="D49" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="E49" s="10" t="s">
+      <c r="E49" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="F49" s="10">
+      <c r="F49" s="9">
         <v>595</v>
       </c>
       <c r="G49" s="3" t="s">
@@ -11222,10 +11216,10 @@
       <c r="D50" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="E50" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="F50" s="10">
+      <c r="F50" s="9">
         <v>595</v>
       </c>
       <c r="G50" s="3" t="s">
@@ -11275,10 +11269,10 @@
       <c r="D51" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="E51" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="F51" s="10">
+      <c r="F51" s="9">
         <v>595</v>
       </c>
       <c r="G51" s="3" t="s">
@@ -11372,10 +11366,10 @@
       <c r="D53" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="E53" s="10" t="s">
+      <c r="E53" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="F53" s="10">
+      <c r="F53" s="9">
         <v>595</v>
       </c>
       <c r="G53" s="3" t="s">
@@ -11416,10 +11410,10 @@
       <c r="D54" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F54" s="10">
+      <c r="F54" s="9">
         <v>7320</v>
       </c>
       <c r="G54" s="3"/>
@@ -11452,10 +11446,10 @@
       <c r="D55" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="E55" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F55" s="10">
+      <c r="F55" s="9">
         <v>7320</v>
       </c>
       <c r="G55" s="3"/>
@@ -11497,10 +11491,10 @@
       <c r="D56" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="E56" s="10" t="s">
+      <c r="E56" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F56" s="10">
+      <c r="F56" s="9">
         <v>7320</v>
       </c>
       <c r="G56" s="3"/>
@@ -11542,10 +11536,10 @@
       <c r="D57" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="E57" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F57" s="10">
+      <c r="F57" s="9">
         <v>7320</v>
       </c>
       <c r="G57" s="3"/>
@@ -11587,10 +11581,10 @@
       <c r="D58" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E58" s="10" t="s">
+      <c r="E58" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F58" s="10">
+      <c r="F58" s="9">
         <v>7320</v>
       </c>
       <c r="G58" s="3"/>
@@ -11632,10 +11626,10 @@
       <c r="D59" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="E59" s="10" t="s">
+      <c r="E59" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F59" s="10">
+      <c r="F59" s="9">
         <v>7320</v>
       </c>
       <c r="G59" s="3"/>
@@ -11668,10 +11662,10 @@
       <c r="D60" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="E60" s="10" t="s">
+      <c r="E60" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="F60" s="10">
+      <c r="F60" s="9">
         <v>7320</v>
       </c>
       <c r="G60" s="3"/>
@@ -11754,10 +11748,10 @@
       <c r="D62" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="E62" s="10" t="s">
+      <c r="E62" s="9" t="s">
         <v>529</v>
       </c>
-      <c r="F62" s="10">
+      <c r="F62" s="9">
         <v>605</v>
       </c>
       <c r="G62" s="3" t="s">
@@ -11977,10 +11971,10 @@
       <c r="D67" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="E67" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="F67" s="10">
+      <c r="F67" s="9">
         <v>650</v>
       </c>
       <c r="G67" s="3" t="s">
@@ -12018,10 +12012,10 @@
       <c r="D68" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E68" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="F68" s="10">
+      <c r="F68" s="9">
         <v>650</v>
       </c>
       <c r="G68" s="3" t="s">
@@ -12059,10 +12053,10 @@
       <c r="D69" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="E69" s="10" t="s">
+      <c r="E69" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="F69" s="10">
+      <c r="F69" s="9">
         <v>650</v>
       </c>
       <c r="G69" s="3" t="s">
@@ -12106,10 +12100,10 @@
       <c r="D70" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="E70" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="F70" s="10">
+      <c r="F70" s="9">
         <v>650</v>
       </c>
       <c r="G70" s="3" t="s">
@@ -12147,10 +12141,10 @@
       <c r="D71" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="E71" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="F71" s="10">
+      <c r="F71" s="9">
         <v>650</v>
       </c>
       <c r="G71" s="3" t="s">
@@ -12232,10 +12226,10 @@
       <c r="D73" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="E73" s="10" t="s">
+      <c r="E73" s="9" t="s">
         <v>531</v>
       </c>
-      <c r="F73" s="10">
+      <c r="F73" s="9">
         <v>656</v>
       </c>
       <c r="G73" s="3" t="s">
@@ -12276,10 +12270,10 @@
       <c r="D74" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="E74" s="10" t="s">
+      <c r="E74" s="9" t="s">
         <v>531</v>
       </c>
-      <c r="F74" s="10">
+      <c r="F74" s="9">
         <v>656</v>
       </c>
       <c r="G74" s="3" t="s">

</xml_diff>